<commit_message>
Add Entrée/Plat/Dessert sections to UI and PDF, update Excel with Catégories sheet
Agent-Logs-Url: https://github.com/LinoVation1312/valise-aux-epices/sessions/a6721e81-1e7e-4f0f-81c1-9f6793f4d40c

Co-authored-by: LinoVation1312 <158364911+LinoVation1312@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/menu_actuel.xlsx
+++ b/menu_actuel.xlsx
@@ -7,31 +7,32 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Poulet Basquaise" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Blanquette de Veau" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Boeuf Bourguignon" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lasagnes Bolognaise" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Risotto aux Champignons" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Hachis Parmentier" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Curry de Pois Chiches" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Tartiflette" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Quiche Lorraine" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Chili con Carne" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Poulet Coco Curry" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gratin Dauphinois" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Couscous Express" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Tacos au Poulet" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Ratatouille" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Pâtes Carbonara" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Saumon Teriyaki" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Moussaka" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Fajitas au Boeuf" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Wok Nouilles Crevettes" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Burger Maison" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Salade César" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Tajine Poulet Citron" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Paella Express" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Gnocchis Pesto Tomates" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Catégories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Poulet Basquaise" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Blanquette de Veau" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Boeuf Bourguignon" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lasagnes Bolognaise" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Risotto aux Champignons" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Hachis Parmentier" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Curry de Pois Chiches" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Tartiflette" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Quiche Lorraine" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Chili con Carne" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Poulet Coco Curry" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Gratin Dauphinois" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Couscous Express" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Tacos au Poulet" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Ratatouille" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Pâtes Carbonara" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Saumon Teriyaki" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Moussaka" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Fajitas au Boeuf" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Wok Nouilles Crevettes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Burger Maison" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Salade César" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Tajine Poulet Citron" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Paella Express" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Gnocchis Pesto Tomates" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,98 +450,318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ingrédient</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Quantité</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Unité</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>Poulet Basquaise</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Plat</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Poivron rouge</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>Blanquette de Veau</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plat</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tomate</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>Boeuf Bourguignon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plat</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>Lasagnes Bolognaise</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plat</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gousse d'ail</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>Risotto aux Champignons</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hachis Parmentier</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Curry de Pois Chiches</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tartiflette</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Quiche Lorraine</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Entrée</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Chili con Carne</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Poulet Coco Curry</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gratin Dauphinois</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Couscous Express</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tacos au Poulet</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ratatouille</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Entrée</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pâtes Carbonara</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saumon Teriyaki</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Moussaka</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fajitas au Boeuf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Wok Nouilles Crevettes</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Burger Maison</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Salade César</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Entrée</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tajine Poulet Citron</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Paella Express</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plat</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Gnocchis Pesto Tomates</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plat</t>
         </is>
       </c>
     </row>
@@ -578,26 +799,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Pâte brisée</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Haricots rouges</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -608,45 +829,45 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Épices Chili</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sachet(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -684,45 +905,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Viande hachée</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
+          <t>Haricots rouges</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Poudre de curry</t>
+          <t>Tomates concassées</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -744,15 +965,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Épices Chili</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>sachet(s)</t>
         </is>
       </c>
     </row>
@@ -790,26 +1011,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Lait de coco</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -820,26 +1041,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crème liquide</t>
+          <t>Poudre de curry</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gousse d'ail</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -850,15 +1071,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Noix de muscade</t>
+          <t>Riz</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pincée(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -896,75 +1117,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Semoule</t>
+          <t>Pomme de terre</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Merguez</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Légumes à couscous</t>
+          <t>Crème liquide</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>600</v>
+        <v>50</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pois chiches</t>
+          <t>Gousse d'ail</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Épices Ras el Hanout</t>
+          <t>Noix de muscade</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pincée(s)</t>
         </is>
       </c>
     </row>
@@ -1002,75 +1223,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Galettes tortillas</t>
+          <t>Semoule</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>300</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Merguez</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>8</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Poivron</t>
+          <t>Légumes à couscous</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>600</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oignon rouge</t>
+          <t>Pois chiches</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Épices mexicaines</t>
+          <t>Épices Ras el Hanout</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sachet(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
@@ -1108,11 +1329,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Courgette</t>
+          <t>Galettes tortillas</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1123,15 +1344,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aubergine</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1153,11 +1374,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Oignon rouge</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1168,7 +1389,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Épices mexicaines</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1176,7 +1397,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>sachet(s)</t>
         </is>
       </c>
     </row>
@@ -1214,41 +1435,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Spaghetti</t>
+          <t>Courgette</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>400</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Guanciale ou Lardons</t>
+          <t>Aubergine</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Poivron</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1259,22 +1480,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pecorino ou Parmesan</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Poivre noir</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1282,7 +1503,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pincée(s)</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1320,56 +1541,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pavé de saumon</t>
+          <t>Spaghetti</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
+          <t>Guanciale ou Lardons</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Miel</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
+          <t>Pecorino ou Parmesan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1380,7 +1601,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Brocoli</t>
+          <t>Poivre noir</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1388,7 +1609,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>pincée(s)</t>
         </is>
       </c>
     </row>
@@ -1426,11 +1647,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aubergine</t>
+          <t>Pavé de saumon</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1441,60 +1662,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée (agneau ou boeuf)</t>
+          <t>Sauce soja</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500</v>
+        <v>10</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sauce tomate</t>
+          <t>Miel</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lait (béchamel)</t>
+          <t>Riz basmati</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fromage râpé</t>
+          <t>Brocoli</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1532,11 +1753,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Galettes tortillas</t>
+          <t>Aubergine</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1547,11 +1768,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Boeuf (bavette)</t>
+          <t>Viande hachée (agneau ou boeuf)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1562,45 +1783,45 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Poivron mix</t>
+          <t>Sauce tomate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Lait (béchamel)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Épices Fajitas</t>
+          <t>Fromage râpé</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sachet(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1638,26 +1859,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viande de veau</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>800</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Poivron rouge</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1668,45 +1889,45 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Champignon de Paris</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>250</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Gousse d'ail</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cube(s)</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1744,22 +1965,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nouilles asiatiques</t>
+          <t>Galettes tortillas</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>250</v>
+        <v>8</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Crevettes décortiquées</t>
+          <t>Boeuf (bavette)</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1774,11 +1995,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Poivron mix</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1789,22 +2010,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Brocoli</t>
+          <t>Épices Fajitas</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1812,7 +2033,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>sachet(s)</t>
         </is>
       </c>
     </row>
@@ -1850,41 +2071,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pain burger</t>
+          <t>Nouilles asiatiques</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>250</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Steak haché</t>
+          <t>Crevettes décortiquées</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cheddar en tranches</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1895,26 +2116,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Salade</t>
+          <t>Sauce soja</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Brocoli</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1956,11 +2177,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Salade Romaine</t>
+          <t>Pain burger</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1971,11 +2192,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Steak haché</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1986,45 +2207,45 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Croûtons</t>
+          <t>Cheddar en tranches</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Salade</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sauce César</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pot</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2062,11 +2283,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cuisse de poulet</t>
+          <t>Salade Romaine</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2077,7 +2298,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Citron confit</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2092,7 +2313,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Olives vertes</t>
+          <t>Croûtons</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2107,22 +2328,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Épices Tajine</t>
+          <t>Sauce César</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2130,7 +2351,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pot</t>
         </is>
       </c>
     </row>
@@ -2168,37 +2389,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Riz à paella</t>
+          <t>Cuisse de poulet</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>300</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Crevettes</t>
+          <t>Citron confit</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Chorizo</t>
+          <t>Olives vertes</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2213,22 +2434,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Petit pois</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Safran ou Spigol</t>
+          <t>Épices Tajine</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2236,7 +2457,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>dose</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
@@ -2274,6 +2495,112 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Riz à paella</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>300</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Crevettes</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Chorizo</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Petit pois</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Safran ou Spigol</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>Gnocchis</t>
         </is>
       </c>
@@ -2380,7 +2707,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viande de boeuf</t>
+          <t>Viande de veau</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2395,60 +2722,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vin rouge</t>
+          <t>Champignon de Paris</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Bouillon de volaille</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cube(s)</t>
         </is>
       </c>
     </row>
@@ -2486,11 +2813,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Viande de boeuf</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2501,60 +2828,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Feuilles de lasagne</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sauce tomate</t>
+          <t>Vin rouge</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gruyère râpé</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2592,11 +2919,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Riz Arborio</t>
+          <t>Viande hachée</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2607,26 +2934,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Champignons</t>
+          <t>Feuilles de lasagne</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300</v>
+        <v>12</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Sauce tomate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>80</v>
+        <v>500</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2637,30 +2964,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Gruyère râpé</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -2698,11 +3025,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Riz Arborio</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2713,11 +3040,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
+          <t>Champignons</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2728,30 +3055,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Beurre</t>
+          <t>Bouillon de volaille</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>L</t>
         </is>
       </c>
     </row>
@@ -2804,11 +3131,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pois chiches (conserve)</t>
+          <t>Viande hachée</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2819,60 +3146,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
+          <t>Pomme de terre</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>800</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>20</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pâte de curry</t>
+          <t>Beurre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2910,41 +3237,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
+          <t>Pois chiches (conserve)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Reblochon</t>
+          <t>Lait de coco</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Tomates concassées</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2955,7 +3282,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Pâte de curry</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2963,22 +3290,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Riz basmati</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>250</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3343,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pâte brisée</t>
+          <t>Pomme de terre</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -3024,63 +3351,63 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Reblochon</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mise à jour menu via admin (menu juin.ods)
</commit_message>
<xml_diff>
--- a/menu_actuel.xlsx
+++ b/menu_actuel.xlsx
@@ -7,36 +7,41 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Risotto aux Crevettes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Quiche Au Thon" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Poulet Basquaise" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Blanquette de Veau" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Boeuf Bourguignon" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Lasagnes Bolognaise" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Risotto aux Champignons" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Hachis Parmentier" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Curry de Pois Chiches" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Tartiflette" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Quiche Lorraine" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Chili con Carne" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Poulet Coco Curry" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Gratin Dauphinois" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Couscous Express" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Tacos au Poulet" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Ratatouille" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Pâtes Carbonara" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Saumon Teriyaki" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Moussaka" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Fajitas au Boeuf" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Wok Nouilles Crevettes" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Burger Maison" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Salade César" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Tajine Poulet Citron" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Paella Express" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Gnocchis Pesto Tomates" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Mousse au Chocolat" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Banofee" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Mi-Cuit Chocolat" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Taboulé" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dhal de lentilles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lentilles vertes au thym" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Salade de mangue à la thaï" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Ratatouille" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Salade de pâtes tomates et feta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Couscous aux légumes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Risotto forestier" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gratin pâtes tomates confites pesto" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Galettes de carottes au cumin" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Chili sin carne" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Rougail saucisses" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Poulet au curry rouge" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Poulet basquaise" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Lentilles aux saucisses" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Lasagnes au boeuf" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Lapin à la moutarde" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Quiche lorraine" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Filet mignon sauce forestière" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Chili con carne" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Nouilles chinoises au boeuf" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Encornet au curry vert" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Risotto de quinoa aux crevettes" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Crumble poireaux saumon" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Crevettes au lait de coco" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Parmentier de poissons" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Saumon sauce soja" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Fondant au chocolat noir" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Mousse au chocolat" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Tiramisu" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Banana bread" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Cheesecake" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Invisible aux pommes" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="Riz au lait" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Semoule aux raisins" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +458,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -478,11 +483,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz Arborio</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>300</v>
+          <t>Semoule</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -493,37 +500,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes</t>
+          <t>Tomates</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Concombre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Persil</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -531,37 +538,54 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>botte</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Menthe</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>botte</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Petits pois</t>
+          <t>Oignons blancs ou rouges</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Citron</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -587,7 +611,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -612,52 +636,58 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+          <t>Carotte</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Reblochon</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
+          <t>Cumin</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lardons</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>200</v>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Farine</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -665,22 +695,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>15</v>
+          <t>Coriandre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>bouquet(s)</t>
         </is>
       </c>
     </row>
@@ -706,7 +738,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -731,26 +763,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pâte brisée</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+          <t>Haricots rouges</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lardons</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>200</v>
+          <t>Tomates concassées</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -761,11 +797,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oeuf</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -776,30 +814,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lait</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>20</v>
+          <t>Épices Chili</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>sachet(s)</t>
         </is>
       </c>
     </row>
@@ -814,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -850,11 +892,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>500</v>
+          <t>Saucisses fumées</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -865,11 +909,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Haricots rouges</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>400</v>
+          <t>Tomates concassées</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -880,45 +926,81 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>400</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
+          <t>Ail</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>gousse(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Chili</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Curcuma</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>sachet(s)</t>
+          <t>c.à.s</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Thym</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>c.à.s</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Riz Basmati</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>250</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -933,7 +1015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -972,12 +1054,14 @@
           <t>Filet de poulet</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>4</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -987,8 +1071,10 @@
           <t>Lait de coco</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>40</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -999,11 +1085,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poudre de curry</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+          <t>Pâte de curry rouge</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1017,8 +1105,10 @@
           <t>Oignon</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>1</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1029,15 +1119,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riz</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>250</v>
+          <t>Riz basmati</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,7 +1170,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1088,15 +1195,100 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>patate</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
+          <t>Filet de poulet</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce</t>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Poivron rouge</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tomate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gousse d'ail</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Riz</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1147,11 +1339,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Semoule</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>300</v>
+          <t>Lentilles vertes</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1162,11 +1356,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Merguez</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>8</v>
+          <t>Saucisses</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1177,43 +1373,64 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Légumes à couscous</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>600</v>
+          <t>Carotte</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pois chiches</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>200</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Ras el Hanout</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Bouillon de volaille</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cube(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Thym</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>c.à.s</t>
         </is>
@@ -1230,7 +1447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1266,75 +1483,128 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Galettes tortillas</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>8</v>
+          <t>Viande hachée</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>400</v>
+          <t>Feuilles de lasagne</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivron</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+          <t>Sauce tomate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon rouge</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices mexicaines</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Gruyère râpé</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>50</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>sachet(s)</t>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1360,7 +1630,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1385,11 +1655,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Courgette</t>
+          <t>Cuisse de Lapin</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1400,41 +1670,45 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aubergine</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
+          <t>Moutarde</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivron</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tomate</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>4</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1445,13 +1719,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Tagliatelles</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>600</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carottes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -1468,7 +1757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1504,26 +1793,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spaghetti</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>400</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Guanciale ou Lardons</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>200</v>
+          <t>Lardons</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1537,8 +1830,10 @@
           <t>Oeuf</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>4</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1549,30 +1844,64 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pecorino ou Parmesan</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>100</v>
+          <t>Crème fraîche</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Poivre noir</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pincée(s)</t>
+          <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>c.à.s</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fromage rapé</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1598,7 +1927,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1623,75 +1952,100 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pavé de saumon</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
+          <t>Filet mignon de porc</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>10</v>
+          <t>Champignons</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Miel</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+          <t>Crème fraîche</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>250</v>
+          <t>Échalote</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brocoli</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Grenailles</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>500</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1717,7 +2071,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1742,86 +2096,96 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pâte brisée</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+          <t>Lentilles corail</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Thon</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>200</v>
+          <t>Lait de coco</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oeuf</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
+          <t>Tomates concassées</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
+          <t>Curry</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lait</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>20</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fromage rapé</t>
+          <t>Riz Basmati</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1840,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1876,26 +2240,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aubergine</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
+          <t>Viande hachée de bœuf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Viande hachée (agneau ou boeuf)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>500</v>
+          <t>Haricots rouges</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1906,11 +2274,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sauce tomate</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>400</v>
+          <t>Tomates concassées</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1921,28 +2291,62 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lait (béchamel)</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fromage râpé</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>100</v>
+          <t>Épices Chili</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>sachet(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Riz </t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>250</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -1959,7 +2363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1995,26 +2399,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Galettes tortillas</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>8</v>
+          <t>Nouilles asiatiques</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Boeuf (bavette)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>400</v>
+          <t>Boeuf (rumsteack ou bavette)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2025,26 +2433,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivron mix</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
+          <t>Sauce soja</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2055,15 +2467,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Fajitas</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Brocoli</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>sachet(s)</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Coriandre</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>bouquet</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2114,11 +2558,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nouilles asiatiques</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>250</v>
+          <t>Encornets</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2129,58 +2575,81 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes décortiquées</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>400</v>
+          <t>Lait de coco</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Carotte</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+          <t>Pâte de curry vert</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brocoli</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Riz basmati</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Poivrons</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -2197,7 +2666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2208,7 +2677,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2233,56 +2702,64 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pain burger</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
+          <t>Quinoa</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Steak haché</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
+          <t>Crevettes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cheddar en tranches</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
+          <t>Bouillon de légumes</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Salade</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2293,13 +2770,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tomate</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Parmesan</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Courgettes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -2327,7 +2821,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2352,26 +2846,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Salade Romaine</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+          <t>Pavé de saumon</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
+          <t>Poireaux</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2382,11 +2880,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Croûtons</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100</v>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2397,11 +2897,13 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parmesan</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2412,15 +2914,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sauce César</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Crème fraîche</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pot</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2446,7 +2950,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2471,75 +2975,100 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cuisse de poulet</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
+          <t>Crevettes</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Citron confit</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
+          <t>Lait de coco</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Olives vertes</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100</v>
+          <t>Citron vert</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
+          <t>Ail</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>gousse(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Tajine</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
+          <t>Riz basmati</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carottes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2554,7 +3083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2590,11 +3119,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz à paella</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>300</v>
+          <t>Filets de poisson blanc</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2605,11 +3136,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>200</v>
+          <t>Pomme de terre</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2620,26 +3153,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chorizo</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100</v>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Petit pois</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>100</v>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2650,15 +3187,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Safran ou Spigol</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Chapelure</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Persil</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>dose</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>botte</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ail</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>gousse(s)</t>
         </is>
       </c>
     </row>
@@ -2684,7 +3253,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2709,56 +3278,64 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gnocchis</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>600</v>
+          <t>Pavé de saumon</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pesto vert</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>150</v>
+          <t>Sauce soja</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates cerises</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>250</v>
+          <t>Miel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parmesan</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>Riz basmati</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2769,15 +3346,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pignons de pin</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>30</v>
+          <t>Brocoli</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2831,8 +3410,10 @@
           <t>Chocolat noir</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>200</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2843,56 +3424,64 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oeuf</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sucre</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>50</v>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème liquide</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Beurre</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>30</v>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2911,7 +3500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2947,60 +3536,68 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Banane</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
+          <t>Chocolat noir</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Caramel au beurre salé</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>200</v>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crème liquide entière</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>30</v>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Biscuits digestifs</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>150</v>
+          <t>Crème liquide</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -3010,25 +3607,12 @@
           <t>Beurre</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>60</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sucre glace</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C8" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -3056,7 +3640,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3081,41 +3665,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
+          <t>Lentilles vertes</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Poivron rouge</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
+          <t>Thym</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>càs</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomate</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
+          <t>Carotte</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3129,8 +3719,10 @@
           <t>Oignon</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>2</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3141,15 +3733,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gousse d'ail</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
+          <t>Bouillon de légumes</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cube(s)</t>
         </is>
       </c>
     </row>
@@ -3200,11 +3794,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chocolat noir</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>150</v>
+          <t>Biscuits à la cuillère</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3215,11 +3811,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Beurre</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>100</v>
+          <t>Mascarpone</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3233,8 +3831,10 @@
           <t>Oeuf</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>4</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3245,28 +3845,688 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sucre</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>80</v>
+          <t>Café fort</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Banane mûre</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Farine</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>250</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>85</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Oeufs</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>160</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Levure</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>càc</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Biscuits speculoos</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fromage blanc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Crème fraîche</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>125</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>càs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Oeufs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Citron vert</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pomme</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>130</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Riz rond</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sucre vanillé</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>sachet</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>càs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Semoule fine</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Raisins secs</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -3283,7 +4543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3294,7 +4554,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3319,26 +4579,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande de veau</t>
+          <t>Mangue verte (dure)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>800</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Carottes</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3349,45 +4609,75 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Champignon de Paris</t>
+          <t>Coriandre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>botte</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Gingembre</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>racine</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Cacahuètes</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sauce soja</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>càs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Citron vert</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>cube(s)</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -3402,7 +4692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3413,7 +4703,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3438,56 +4728,64 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande de boeuf</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>800</v>
+          <t>Courgette</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lardons</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>150</v>
+          <t>Aubergine</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vin rouge</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>50</v>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Carotte</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
+          <t>Tomate</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3501,12 +4799,29 @@
           <t>Oignon</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>2</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Herbes de Provence</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>càs</t>
         </is>
       </c>
     </row>
@@ -3521,7 +4836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,7 +4847,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3557,11 +4872,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Pâtes fusili ou penne</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3572,11 +4887,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Feuilles de lasagne</t>
+          <t>Tomates</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3587,11 +4902,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sauce tomate</t>
+          <t>Feta</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3602,28 +4917,47 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lait</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>Concombre</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gruyère râpé</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Basilic</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>botte</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Olives noires</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>100</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -3640,7 +4974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3676,11 +5010,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz Arborio</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>300</v>
+          <t>Semoule</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3691,26 +5027,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Champignons</t>
+          <t>Poivrons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parmesan</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>80</v>
+          <t>Pois chiches</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3721,28 +5059,77 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
+          <t>Épices Ras el Hanout</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Bouillon de légumes</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cube(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Courgettes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Oignon</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carottes</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -3770,7 +5157,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3795,11 +5182,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>500</v>
+          <t>Riz Arborio</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3810,11 +5199,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>800</v>
+          <t>Champignons</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3825,30 +5216,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lait</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>20</v>
+          <t>Parmesan</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Beurre</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>Bouillon de légumes</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>L</t>
         </is>
       </c>
     </row>
@@ -3858,8 +5253,10 @@
           <t>Oignon</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3914,11 +5311,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pois chiches (conserve)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>400</v>
+          <t>Pâtes</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3929,26 +5328,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>40</v>
+          <t>Tomates cerises confites</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>400</v>
+          <t>Pesto vert</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3959,30 +5362,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pâte de curry</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
+          <t>Fromage râpé</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>250</v>
+          <t>Crème fraîche</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour menu via admin (menu_actuel.xlsx)
</commit_message>
<xml_diff>
--- a/menu_actuel.xlsx
+++ b/menu_actuel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lconord.LYD\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19F2BEE1-6AD5-4B2C-98F3-CB8E8C1D841B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A4C4FD-360E-4012-9420-7A22E0C90DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Taboulé" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,6 @@
     <sheet name="Semoule aux raisins" sheetId="35" r:id="rId35"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -864,7 +863,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3597,7 +3596,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour menu via admin (menu septembre.ods)
</commit_message>
<xml_diff>
--- a/menu_actuel.xlsx
+++ b/menu_actuel.xlsx
@@ -7,33 +7,39 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pancakes épinards saumon" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Blanquette de Veau" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Clafoutis jambon courgettes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Risotto aux Crevettes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Quiche Au Thon" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Tortilla quiche au jambon" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Crumble salé au poulet" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Poulet Basquaise" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Poulet miel soja " sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lasagnes Bolognaise" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Risotto aux Champignons" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Hachis Parmentier" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Chili con Carne" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Curry de Pois Chiches" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Tartiflette" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Quiche Lorraine" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Poulet Coco Curry" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Ratatouille" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Pâtes Carbonara" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Saumon Teriyaki" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Wok Nouilles Crevettes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Salade César" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Tajine Poulet Citron" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Paella Express" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Gnocchis Pesto Tomates" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Mousse au Chocolat" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Mi-Cuit Chocolat" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Poke bowl au saumon" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Salade de pois chiches- tomates confites-feta " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Croustade aux pommes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Riz au lait" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cookies au chocolat" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Crumble pommes fraises" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Pancakes épinards saumon" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Blanquette de Veau" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Clafoutis jambon courgettes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Risotto aux Crevettes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Quiche Au Thon" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Tortilla quiche au jambon" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crumble salé au poulet" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Poulet Basquaise" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Poulet miel soja " sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Lasagnes Bolognaise" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Risotto aux Champignons" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Hachis Parmentier" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Chili con Carne" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Curry de Pois Chiches" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Tartiflette" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Quiche Lorraine" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Poulet Coco Curry" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Ratatouille" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Pâtes Carbonara" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Saumon Teriyaki" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Wok Nouilles Crevettes" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Salade César" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Tajine Poulet Citron" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Paella Express" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gnocchis Pesto Tomates" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Mousse au Chocolat" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Mi-Cuit Chocolat" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,7 +456,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -475,26 +481,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Farine</t>
+          <t>Tomates</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oeufs</t>
+          <t>Poivrons rouges</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -505,60 +511,60 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Concombre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Epinards frais</t>
+          <t>Coriandre</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>botte</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Levure</t>
+          <t>Riz</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>càc</t>
+          <t xml:space="preserve">g </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Oignons rouges</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -569,41 +575,71 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>tranche(s)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fromage blanc</t>
+          <t>Citron vert</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ciboulette</t>
+          <t xml:space="preserve">Avocat </t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Maïs</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>botte</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>boîte</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sauce soja</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -618,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +665,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -654,11 +690,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Riz Arborio</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -669,26 +705,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Feuilles de lasagne</t>
+          <t>Crevettes</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sauce tomate</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -699,58 +735,43 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Bouillon de volaille</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gruyère râpé</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Beurre</t>
+          <t>Petits pois</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>100</v>
       </c>
       <c r="C8" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Farine</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>100</v>
-      </c>
-      <c r="C9" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -767,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -778,7 +799,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -803,26 +824,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz Arborio</t>
+          <t>Pâte brisée</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Champignons</t>
+          <t>Thon</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -833,45 +854,60 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fromage rapé</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -886,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -897,7 +933,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -922,75 +958,105 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Tortilla de blé</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>grande(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
+          <t>Oeufs</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>800</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Jambon</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t xml:space="preserve">g </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Beurre</t>
+          <t>Poivron</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Emmental</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ml</t>
         </is>
       </c>
     </row>
@@ -1041,11 +1107,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande hachée</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1056,75 +1122,75 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Haricots rouges</t>
+          <t>Aubergine</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>400</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Farine</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Chili</t>
+          <t>Chapelure</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>sachet(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Poivron</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1150,7 +1216,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1175,52 +1241,52 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pois chiches (conserve)</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
+          <t>Poivron rouge</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates concassées</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>400</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pâte de curry</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1228,52 +1294,37 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
+          <t>Gousse d'ail</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Riz</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>240</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Coriandre</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>bouquet</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1324,75 +1375,75 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pomme de terre</t>
+          <t>Filet de Poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>600</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Reblochon</t>
+          <t>Riz</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>220</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Poivrons</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Miel</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Soja</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>ml</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1418,7 +1469,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1443,56 +1494,56 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pâte brisée</t>
+          <t>Viande hachée</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lardons</t>
+          <t>Feuilles de lasagne</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>12</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Sauce tomate</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>500</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1503,28 +1554,43 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Gruyère râpé</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Emmental</t>
+          <t>Beurre</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -1552,7 +1618,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1577,52 +1643,52 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Riz Arborio</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lait de coco</t>
+          <t>Champignons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poudre de curry</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Bouillon de volaille</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1630,22 +1696,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1737,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1696,60 +1762,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Courgette</t>
+          <t>Viande hachée</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>500</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aubergine</t>
+          <t>Pomme de terre</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>800</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivron</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Beurre</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1815,11 +1881,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spaghetti</t>
+          <t>Viande hachée</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1830,11 +1896,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Lardons</t>
+          <t>Haricots rouges</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1845,43 +1911,58 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crème</t>
+          <t>Tomates concassées</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>400</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pecorino ou Parmesan</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Épices Chili</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>sachet(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -1909,7 +1990,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -1934,11 +2015,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Viande de veau</t>
+          <t>Pois chiches</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1949,26 +2030,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Tomates confites</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Champignon de Paris</t>
+          <t>Feta</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1979,22 +2060,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Menthe</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>bouquet</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Oignons rouges</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2002,33 +2083,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cube(s)</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Concombre</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>240</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Poireau</t>
+          <t>Citron</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2047,7 +2128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2058,7 +2139,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2083,26 +2164,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pavé de saumon</t>
+          <t>Pois chiches (conserve)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
+          <t>Lait de coco</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2113,45 +2194,75 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Miel</t>
+          <t>Tomates concassées</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.à.s</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Riz basmati</t>
+          <t>Pâte de curry</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brocoli</t>
+          <t>Riz basmati</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>250</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Coriandre</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>bouquet</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2288,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2202,75 +2313,75 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nouilles asiatiques</t>
+          <t>Pomme de terre</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes décortiquées</t>
+          <t>Reblochon</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Carotte</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sauce soja</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brocoli</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2321,7 +2432,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Salade Romaine</t>
+          <t>Pâte brisée</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2336,105 +2447,75 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Lardons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Croûtons</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sauce César</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pot</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Emmental</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Tomate</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Concombre</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2485,7 +2566,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cuisse de poulet</t>
+          <t>Filet de poulet</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2500,30 +2581,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Citron confit</t>
+          <t>Lait de coco</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Olives vertes</t>
+          <t>Poudre de curry</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2615,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2545,60 +2626,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Épices Tajine</t>
+          <t>Riz</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>c.à.s</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Couscous</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>500</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Courgette</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Poivron</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -2613,7 +2649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2624,7 +2660,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Plat végé</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2649,103 +2685,73 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz à paella</t>
+          <t>Courgette</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300</v>
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes</t>
+          <t>Aubergine</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chorizo</t>
+          <t>Poivron</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Petit pois</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Safran ou Spigol</t>
+          <t>Oignon</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Cube ou bouillon</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
         <is>
           <t>pièce(s)</t>
         </is>
@@ -2762,7 +2768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2773,7 +2779,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat végé</t>
+          <t>Plat viande</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2798,11 +2804,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gnocchis</t>
+          <t>Spaghetti</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2813,11 +2819,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pesto vert</t>
+          <t xml:space="preserve"> Lardons</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2828,30 +2834,45 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomates confites</t>
+          <t>Crème</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>250</v>
+        <v>20</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parmesan</t>
+          <t>Pecorino ou Parmesan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2898,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Dessert</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -2902,75 +2923,75 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chocolat noir</t>
+          <t>Pavé de saumon</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Sauce soja</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sucre</t>
+          <t>Miel</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>c.à.s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème liquide</t>
+          <t>Riz basmati</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Beurre</t>
+          <t>Brocoli</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -2996,7 +3017,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Dessert</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3021,11 +3042,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chocolat noir</t>
+          <t>Nouilles asiatiques</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3036,11 +3057,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Beurre</t>
+          <t>Crevettes décortiquées</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3051,11 +3072,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3066,30 +3087,358 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sucre</t>
+          <t>Sauce soja</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Farine</t>
+          <t>Brocoli</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Entrée</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Salade Romaine</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Filet de poulet</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Croûtons</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Parmesan</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sauce César</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pot</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tomate</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Concombre</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Plat viande</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cuisse de poulet</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Citron confit</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Olives vertes</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Épices Tajine</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>c.à.s</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Couscous</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>500</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Courgette</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Poivron</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -3104,6 +3453,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pomme</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pâte Filo</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>feuille(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -3115,7 +3570,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3140,22 +3595,171 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Courgettes</t>
+          <t>Riz à paella</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>300</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jambon</t>
+          <t>Crevettes</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>200</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Chorizo</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Petit pois</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Safran ou Spigol</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cube ou bouillon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Oignon</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Plat végé</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gnocchis</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pesto vert</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3170,11 +3774,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Feta</t>
+          <t>Tomates confites</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3185,58 +3789,251 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oeufs</t>
+          <t>Parmesan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Chocolat noir</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Crème liquide</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Beurre</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ml</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Emmental</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>50</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Catégorie :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dessert</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingrédient</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Chocolat noir</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Beurre</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Oeuf</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>80</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Farine</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>60</v>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -3253,7 +4050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3264,7 +4061,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat poisson</t>
+          <t>Dessert</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3289,11 +4086,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Riz Arborio</t>
+          <t>Riz rond</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3304,75 +4101,47 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crevettes</t>
+          <t>Sucre vanillé</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>sachet</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parmesan</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>80</v>
+          <t>Lait</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bouillon de volaille</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Oignon</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Petits pois</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>g</t>
+          <t>càs</t>
         </is>
       </c>
     </row>
@@ -3398,7 +4167,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Dessert</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3423,26 +4192,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pâte brisée</t>
+          <t>Chocolat</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Thon</t>
+          <t>Beurre</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3453,60 +4222,60 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oeuf</t>
+          <t>Farine</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>150</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crème fraîche</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lait</t>
+          <t>Oeuf</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cl</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fromage rapé</t>
+          <t>Levure</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>càc</t>
         </is>
       </c>
     </row>
@@ -3521,7 +4290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,7 +4301,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Dessert</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3557,105 +4326,75 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tortilla de blé</t>
+          <t>Pommes</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>grande(s)</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oeufs</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jambon</t>
+          <t>Fraises</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">g </t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Poivron</t>
+          <t>Farine</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Beurre</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>130</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Emmental</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">g </t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Lait</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>100</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
     </row>
@@ -3670,7 +4409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3681,7 +4420,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Plat poisson</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3706,11 +4445,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Farine</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3721,11 +4460,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aubergine</t>
+          <t>Oeufs</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3736,26 +4475,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>ml</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Farine</t>
+          <t>Epinards frais</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3766,15 +4505,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Chapelure</t>
+          <t>Levure</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>càc</t>
         </is>
       </c>
     </row>
@@ -3790,6 +4529,51 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saumon fumé</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>200</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fromage blanc</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ciboulette</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>botte</t>
         </is>
       </c>
     </row>
@@ -3804,7 +4588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3840,26 +4624,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de poulet</t>
+          <t>Viande de veau</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>800</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Poivron rouge</t>
+          <t>Carotte</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3870,45 +4654,45 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomate</t>
+          <t>Champignon de Paris</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>250</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oignon</t>
+          <t>Crème fraîche</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gousse d'ail</t>
+          <t>Bouillon de volaille</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>cube(s)</t>
         </is>
       </c>
     </row>
@@ -3924,6 +4708,21 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Poireau</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
@@ -3938,7 +4737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3949,7 +4748,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plat viande</t>
+          <t>Entrée</t>
         </is>
       </c>
       <c r="C1" t="inlineStr"/>
@@ -3974,26 +4773,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filet de Poulet</t>
+          <t>Courgettes</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>600</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Jambon</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -4004,45 +4803,75 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poivrons</t>
+          <t>Feta</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pièce(s)</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Miel</t>
+          <t>Oeufs</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pièce(s)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Soja</t>
+          <t>Lait</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>200</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Emmental</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Farine</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>60</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ml</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
     </row>

</xml_diff>